<commit_message>
feat: update catalog handling to support multiple triggers and improve documentation
</commit_message>
<xml_diff>
--- a/public/plantillas/pilo/pilo-capciosas.xlsx
+++ b/public/plantillas/pilo/pilo-capciosas.xlsx
@@ -34,7 +34,7 @@
     <comment ref="C1" authorId="0">
       <text>
         <r>
-          <t>Palabras que activan la respuesta, un grupo por línea o separados por |. Todas las palabras del grupo deben estar en la pregunta, en cualquier orden.</t>
+          <t>Palabras que activan la respuesta, separadas por coma, punto y coma, | o una por línea (salario, sueldo, cuánto gana). Si un disparador tiene varias palabras, todas deben estar en la pregunta, en cualquier orden.</t>
         </r>
       </text>
     </comment>
@@ -156,7 +156,7 @@
     <t>Disparadores (obligatoria)</t>
   </si>
   <si>
-    <t>Palabras que activan la respuesta, un grupo por línea o separados por |. Todas las palabras del grupo deben estar en la pregunta, en cualquier orden.</t>
+    <t>Palabras que activan la respuesta, separadas por coma, punto y coma, | o una por línea (salario, sueldo, cuánto gana). Si un disparador tiene varias palabras, todas deben estar en la pregunta, en cualquier orden.</t>
   </si>
   <si>
     <t>Respuesta (obligatoria)</t>

</xml_diff>

<commit_message>
feat: Enhance Pilo catalog functionality with new modal for entries
- Added CatalogModal component for creating and editing catalog entries.
- Implemented automatic key generation for new entries.
- Introduced triggers and keywords extraction for responses.
- Updated catalog parsing to recognize column aliases and generate keys if missing.
- Enhanced tests for catalog parsing and detection of catalog kind.
- Improved CSS styles for modal forms and catalog actions.
- Added permissions for authenticated users to insert and update catalog entries directly.
</commit_message>
<xml_diff>
--- a/public/plantillas/pilo/pilo-capciosas.xlsx
+++ b/public/plantillas/pilo/pilo-capciosas.xlsx
@@ -20,7 +20,7 @@
     <comment ref="A1" authorId="0">
       <text>
         <r>
-          <t>Única y corta: C-001, C-002… Importar otra vez la misma clave la actualiza.</t>
+          <t>Única y corta: C-001, C-002… Si se deja vacía se genera automáticamente. Importar otra vez la misma clave la actualiza.</t>
         </r>
       </text>
     </comment>
@@ -34,7 +34,7 @@
     <comment ref="C1" authorId="0">
       <text>
         <r>
-          <t>Palabras que activan la respuesta, separadas por coma, punto y coma, | o una por línea (salario, sueldo, cuánto gana). Si un disparador tiene varias palabras, todas deben estar en la pregunta, en cualquier orden.</t>
+          <t>Palabras que activan la respuesta, separadas por coma, punto y coma, | o una por línea (salario, sueldo, cuánto gana). Si un disparador tiene varias palabras, todas deben estar en la pregunta, en cualquier orden; no cuentan las de relleno (el, una, eres, usted) y valen plural, femenino y tú o usted (tienes = tiene).</t>
         </r>
       </text>
     </comment>
@@ -147,7 +147,7 @@
     <t>Clave (obligatoria)</t>
   </si>
   <si>
-    <t>Única y corta: C-001, C-002… Importar otra vez la misma clave la actualiza.</t>
+    <t>Única y corta: C-001, C-002… Si se deja vacía se genera automáticamente. Importar otra vez la misma clave la actualiza.</t>
   </si>
   <si>
     <t>Para usted: de qué trata (salarios, vida personal de Pilo…).</t>
@@ -156,7 +156,7 @@
     <t>Disparadores (obligatoria)</t>
   </si>
   <si>
-    <t>Palabras que activan la respuesta, separadas por coma, punto y coma, | o una por línea (salario, sueldo, cuánto gana). Si un disparador tiene varias palabras, todas deben estar en la pregunta, en cualquier orden.</t>
+    <t>Palabras que activan la respuesta, separadas por coma, punto y coma, | o una por línea (salario, sueldo, cuánto gana). Si un disparador tiene varias palabras, todas deben estar en la pregunta, en cualquier orden; no cuentan las de relleno (el, una, eres, usted) y valen plural, femenino y tú o usted (tienes = tiene).</t>
   </si>
   <si>
     <t>Respuesta (obligatoria)</t>

</xml_diff>